<commit_message>
Update subscription billing Excel sheet
</commit_message>
<xml_diff>
--- a/ExcelSheet/Subscription Billing System.xlsx
+++ b/ExcelSheet/Subscription Billing System.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b643115766601192/Desktop/CodeSparks Internship/ExcelSheet/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{C5B584D0-03F7-4CC9-8163-822A2013A825}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="9" documentId="8_{C5B584D0-03F7-4CC9-8163-822A2013A825}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{25B8F2C3-EA1D-47BD-8BC5-4BC35D67440A}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{480AE71A-3966-42F9-A2BF-DC6683A1AD79}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="83" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="36">
   <si>
     <t>UserDetails</t>
   </si>
@@ -124,6 +124,15 @@
   </si>
   <si>
     <t>changeReturned</t>
+  </si>
+  <si>
+    <t>FOREIGN KEY (user_id) REFERENCES users(user_id)</t>
+  </si>
+  <si>
+    <t>FK(userId) references UserDetails(userId)</t>
+  </si>
+  <si>
+    <t>FK(planName) references PlanDetails(planName)</t>
   </si>
 </sst>
 </file>
@@ -544,20 +553,21 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4CDCFDCB-08BB-4072-8017-BFF405A0D906}">
-  <dimension ref="A1:J26"/>
+  <dimension ref="A1:L26"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.5546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9.21875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="24" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="41.109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="20.5546875" customWidth="1"/>
     <col min="7" max="7" width="14.33203125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="9.21875" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="24" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="8" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="42.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -571,7 +581,7 @@
       <c r="I1" s="4"/>
       <c r="J1" s="5"/>
     </row>
-    <row r="2" spans="1:10" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A2" s="2" t="s">
         <v>1</v>
       </c>
@@ -597,7 +607,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>5</v>
       </c>
@@ -619,7 +629,7 @@
       </c>
       <c r="J3" s="1"/>
     </row>
-    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
@@ -641,7 +651,7 @@
       </c>
       <c r="J4" s="1"/>
     </row>
-    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>7</v>
       </c>
@@ -663,7 +673,7 @@
       </c>
       <c r="J5" s="1"/>
     </row>
-    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>8</v>
       </c>
@@ -685,7 +695,7 @@
       </c>
       <c r="J6" s="1"/>
     </row>
-    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>9</v>
       </c>
@@ -707,7 +717,7 @@
       </c>
       <c r="J7" s="1"/>
     </row>
-    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
@@ -722,8 +732,11 @@
         <v>13</v>
       </c>
       <c r="J8" s="1"/>
-    </row>
-    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="L8" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
@@ -739,7 +752,7 @@
       </c>
       <c r="J9" s="1"/>
     </row>
-    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A12" s="3" t="s">
         <v>14</v>
       </c>
@@ -747,7 +760,7 @@
       <c r="C12" s="4"/>
       <c r="D12" s="5"/>
     </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
         <v>1</v>
       </c>
@@ -761,7 +774,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>15</v>
       </c>
@@ -773,7 +786,7 @@
       </c>
       <c r="D14" s="1"/>
     </row>
-    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>16</v>
       </c>
@@ -785,7 +798,7 @@
       </c>
       <c r="D15" s="1"/>
     </row>
-    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
         <v>17</v>
       </c>
@@ -839,7 +852,7 @@
         <v>10</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>23</v>
+        <v>34</v>
       </c>
       <c r="D22" s="1"/>
     </row>
@@ -851,7 +864,7 @@
         <v>11</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>24</v>
+        <v>35</v>
       </c>
       <c r="D23" s="1"/>
     </row>

</xml_diff>

<commit_message>
Add SQLAlchemyORM, dataClass; update Excel sheet and project config
</commit_message>
<xml_diff>
--- a/ExcelSheet/Subscription Billing System.xlsx
+++ b/ExcelSheet/Subscription Billing System.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b643115766601192/Desktop/CodeSparks Internship/ExcelSheet/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="9" documentId="8_{C5B584D0-03F7-4CC9-8163-822A2013A825}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{25B8F2C3-EA1D-47BD-8BC5-4BC35D67440A}"/>
+  <xr:revisionPtr revIDLastSave="14" documentId="8_{C5B584D0-03F7-4CC9-8163-822A2013A825}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C54B548B-8D38-4791-B64D-FD9BAEB9331D}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{480AE71A-3966-42F9-A2BF-DC6683A1AD79}"/>
   </bookViews>
@@ -25,10 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="36">
-  <si>
-    <t>UserDetails</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="80" uniqueCount="33">
   <si>
     <t>Column Name</t>
   </si>
@@ -42,9 +39,6 @@
     <t>Remarks</t>
   </si>
   <si>
-    <t>userId</t>
-  </si>
-  <si>
     <t>name</t>
   </si>
   <si>
@@ -69,70 +63,67 @@
     <t>Not Null</t>
   </si>
   <si>
-    <t>PlanDetails</t>
-  </si>
-  <si>
-    <t>planId</t>
-  </si>
-  <si>
-    <t>planName</t>
-  </si>
-  <si>
-    <t>planPrice</t>
-  </si>
-  <si>
-    <t>SubscriptionDetails</t>
-  </si>
-  <si>
-    <t>subscriptionId</t>
-  </si>
-  <si>
     <t>amount</t>
   </si>
   <si>
-    <t>startDate</t>
-  </si>
-  <si>
     <t>status</t>
   </si>
   <si>
-    <t>FK(UserDetails)</t>
-  </si>
-  <si>
-    <t>FK(PlanDetails)</t>
-  </si>
-  <si>
     <t>date</t>
   </si>
   <si>
     <t>boolean</t>
   </si>
   <si>
-    <t>InvoiceDetails</t>
-  </si>
-  <si>
-    <t>invoiceId</t>
-  </si>
-  <si>
-    <t>payment</t>
-  </si>
-  <si>
-    <t>billingDate</t>
-  </si>
-  <si>
-    <t>FK(SubscriptionDetails)</t>
-  </si>
-  <si>
-    <t>changeReturned</t>
-  </si>
-  <si>
-    <t>FOREIGN KEY (user_id) REFERENCES users(user_id)</t>
-  </si>
-  <si>
-    <t>FK(userId) references UserDetails(userId)</t>
-  </si>
-  <si>
-    <t>FK(planName) references PlanDetails(planName)</t>
+    <t>id</t>
+  </si>
+  <si>
+    <t>price</t>
+  </si>
+  <si>
+    <t>users</t>
+  </si>
+  <si>
+    <t>plans</t>
+  </si>
+  <si>
+    <t>d</t>
+  </si>
+  <si>
+    <t>subscriptions</t>
+  </si>
+  <si>
+    <t>user_id</t>
+  </si>
+  <si>
+    <t>FK(id) references users(id)</t>
+  </si>
+  <si>
+    <t>plan_id</t>
+  </si>
+  <si>
+    <t>FK(id) references plans(id)</t>
+  </si>
+  <si>
+    <t>start_date</t>
+  </si>
+  <si>
+    <t>invoices</t>
+  </si>
+  <si>
+    <t>FK(id) references user(id)</t>
+  </si>
+  <si>
+    <t>change_returned</t>
+  </si>
+  <si>
+    <t>billing_date</t>
+  </si>
+  <si>
+    <t>FK(id) references subscriptions(id)</t>
+  </si>
+  <si>
+    <t>decimal</t>
   </si>
 </sst>
 </file>
@@ -220,10 +211,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="7">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
@@ -235,10 +229,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -553,354 +543,342 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4CDCFDCB-08BB-4072-8017-BFF405A0D906}">
-  <dimension ref="A1:L26"/>
+  <dimension ref="A1:J26"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="12.5546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="9.21875" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="41.109375" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="20.5546875" customWidth="1"/>
-    <col min="7" max="7" width="14.33203125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="42.77734375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="8" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="15.109375" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="9.21875" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="24" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="29.5546875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="8" bestFit="1" customWidth="1"/>
     <col min="12" max="12" width="42.77734375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A1" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1" s="5"/>
+      <c r="C1" s="5"/>
+      <c r="D1" s="6"/>
+      <c r="G1" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="H1" s="5"/>
+      <c r="I1" s="5"/>
+      <c r="J1" s="6"/>
+    </row>
+    <row r="2" spans="1:10" s="3" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="4"/>
-      <c r="C1" s="4"/>
-      <c r="D1" s="5"/>
-      <c r="G1" s="3" t="s">
-        <v>27</v>
-      </c>
-      <c r="H1" s="4"/>
-      <c r="I1" s="4"/>
-      <c r="J1" s="5"/>
-    </row>
-    <row r="2" spans="1:12" s="6" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="2" t="s">
+      <c r="B2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="C2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="2" t="s">
+      <c r="D2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D2" s="2" t="s">
-        <v>4</v>
-      </c>
       <c r="G2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="H2" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="I2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="J2" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="J2" s="2" t="s">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
-        <v>5</v>
+        <v>16</v>
       </c>
       <c r="B3" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>10</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>12</v>
       </c>
       <c r="D3" s="1"/>
       <c r="G3" s="1" t="s">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="H3" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="I3" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="I3" s="1" t="s">
-        <v>12</v>
-      </c>
       <c r="J3" s="1"/>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D4" s="1"/>
       <c r="G4" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="J4" s="1"/>
+    </row>
+    <row r="5" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="H4" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="I4" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="J4" s="1"/>
-    </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A5" s="1" t="s">
-        <v>7</v>
-      </c>
       <c r="B5" s="1" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D5" s="1"/>
       <c r="G5" s="1" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="J5" s="1"/>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B6" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="1" t="s">
-        <v>10</v>
-      </c>
       <c r="C6" s="1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D6" s="1"/>
       <c r="G6" s="1" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="I6" s="1" t="s">
         <v>31</v>
       </c>
       <c r="J6" s="1"/>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B7" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="B7" s="1" t="s">
-        <v>11</v>
-      </c>
       <c r="C7" s="1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D7" s="1"/>
       <c r="G7" s="1" t="s">
         <v>29</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="J7" s="1"/>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
       <c r="B8" s="1"/>
       <c r="C8" s="1"/>
       <c r="D8" s="1"/>
       <c r="G8" s="1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="J8" s="1"/>
-      <c r="L8" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
       <c r="B9" s="1"/>
       <c r="C9" s="1"/>
       <c r="D9" s="1"/>
-      <c r="G9" s="7" t="s">
-        <v>30</v>
-      </c>
-      <c r="H9" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="I9" s="1" t="s">
-        <v>13</v>
-      </c>
       <c r="J9" s="1"/>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A12" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="B12" s="4"/>
-      <c r="C12" s="4"/>
-      <c r="D12" s="5"/>
-    </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A12" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B12" s="5"/>
+      <c r="C12" s="5"/>
+      <c r="D12" s="6"/>
+    </row>
+    <row r="13" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A13" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B13" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B13" s="2" t="s">
+      <c r="C13" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C13" s="2" t="s">
+      <c r="D13" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="D13" s="2" t="s">
+    </row>
+    <row r="14" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A14" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="D14" s="1"/>
+    </row>
+    <row r="15" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A15" s="1" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A14" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="D14" s="1"/>
-    </row>
-    <row r="15" spans="1:12" x14ac:dyDescent="0.3">
-      <c r="A15" s="1" t="s">
-        <v>16</v>
-      </c>
       <c r="B15" s="1" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D15" s="1"/>
     </row>
-    <row r="16" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
         <v>17</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>10</v>
+        <v>32</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D16" s="1"/>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A19" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="B19" s="4"/>
-      <c r="C19" s="4"/>
-      <c r="D19" s="5"/>
+      <c r="A19" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B19" s="5"/>
+      <c r="C19" s="5"/>
+      <c r="D19" s="6"/>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A20" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B20" s="2" t="s">
         <v>1</v>
       </c>
-      <c r="B20" s="2" t="s">
+      <c r="C20" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C20" s="2" t="s">
+      <c r="D20" s="2" t="s">
         <v>3</v>
-      </c>
-      <c r="D20" s="2" t="s">
-        <v>4</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B21" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C21" s="1" t="s">
         <v>10</v>
-      </c>
-      <c r="C21" s="1" t="s">
-        <v>12</v>
       </c>
       <c r="D21" s="1"/>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
-        <v>5</v>
+        <v>22</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>34</v>
+        <v>23</v>
       </c>
       <c r="D22" s="1"/>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
-        <v>16</v>
+        <v>24</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="D23" s="1"/>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>10</v>
+        <v>32</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D24" s="1"/>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
-        <v>21</v>
+        <v>26</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D25" s="1"/>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>26</v>
+        <v>15</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D26" s="1"/>
     </row>

</xml_diff>